<commit_message>
fix: the Excel export kept only the first column (low-memory mode drops a row once the next starts, and pandas writes column by column): rows written whole; rule dates as text
</commit_message>
<xml_diff>
--- a/dataset/3_tax_and_charges_rules/structured/Exchange_and_government_charges_by_date.xlsx
+++ b/dataset/3_tax_and_charges_rules/structured/Exchange_and_government_charges_by_date.xlsx
@@ -22,19 +22,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
-  </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -50,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -58,31 +47,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -381,42 +351,42 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>segment</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>from</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>verified_on</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>to</t>
         </is>
@@ -428,6 +398,36 @@
           <t>delivery</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>S1 and S39 Clearing Charges for delivery: 0; S31 no clearing charge in the delivery calculation of 2018 to 2020</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Zero on Fyers' published tables.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -435,6 +435,41 @@
           <t>futures</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>0.000005</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>S31 futures charge 0.0024% = exchange 0.0019% + clearing 0.0005% in the 2018 calculator</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Earlier years were not researched; the 2018 value is used as a stand-in.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2018-03-03</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -442,8 +477,10 @@
           <t>futures</t>
         </is>
       </c>
-      <c r="B4" s="2">
-        <v>43163</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2018-03-04</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -455,8 +492,10 @@
           <t>S30 Clearing charge: 0.0005% (equity futures); S31 futures total 0.0024% = 0.0019% + 0.0005% in 2018, 2019 and 2020; S1 today: 0.0005%</t>
         </is>
       </c>
-      <c r="E4" s="2">
-        <v>46295</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -480,55 +519,121 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>from</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>to</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>verified_on</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
-        <v>40269</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2019-11-14</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>5.5</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>S7 depository charges at actuals (Fyers page of 2018-09-15)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Rs 5.5 is the amount Fyers' pages show for CDSL from 2019 and is used as a stand-in for earlier years.</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
-        <v>43784</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2019-11-15</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2024-09-30</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>5.5</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>S8 Rs 10 + Rs 5.50 (CDSL Charges); S12 and S13 Rs 5.5 (CDSL Charges)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>CDSL's tariff to DPs was slab-based, from Rs 3.75 to Rs 5.50, before 2024-10-01 (S38 press coverage); Rs 5.5 is what Fyers passed on.</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2">
-        <v>45566</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2024-10-01</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -540,8 +645,10 @@
           <t>S38 Uniform tariff of Rs. 3.50 per debit transaction, effective from October 01, 2024</t>
         </is>
       </c>
-      <c r="E4" s="2">
-        <v>46295</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -565,47 +672,47 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>exchange</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>segment</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>from</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>to</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>verified_on</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -617,6 +724,46 @@
           <t>NSE</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>delivery</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2020-12-31</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0.0000325</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>S25 existing Rs 3.25 each side per lakh of traded value (cash market); S31 and S30 0.00325%</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Confirmed for 2018 to 2020 (Fyers calculator scripts, S31, S30) and for 2020-12-18 (NSE circular S25). The same rate is used back to 2010: earlier NSE rates and any ETF concessions were not researched.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -624,6 +771,46 @@
           <t>NSE</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>delivery</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2021-01-01</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2023-03-31</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.0000345</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>S25 revised Rs 3.45 each side per lakh, applicable with effect from January 01, 2021</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Fyers' published tables of 2022 and 2023 still showed 0.00325%; the NSE first-slab rate is used.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -631,6 +818,41 @@
           <t>NSE</t>
         </is>
       </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>delivery</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2023-04-01</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2024-03-31</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.0000325</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>S26 cash market revised Rs 3.25 each side per lakh, applicable with effect from April 01, 2023</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -638,6 +860,46 @@
           <t>NSE</t>
         </is>
       </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>delivery</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2024-04-01</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2024-09-30</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0.0000322</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>S27 cash market revised Rs 3.22 each side per lakh, applicable with effect from April 01, 2024</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Fyers' notice S14 calls 0.003220% the old charge.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -645,6 +907,46 @@
           <t>NSE</t>
         </is>
       </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>delivery</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2024-10-01</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.0000297</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>S28 Cash Market: Rs. 2.97 each side per lakh of traded value, with effect from October 1, 2024</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Uniform rate under SEBI's true-to-label circular.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -652,6 +954,41 @@
           <t>NSE</t>
         </is>
       </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>delivery</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0.000030699</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>S29 Cash Market transaction charges Rs. 306.99 each side per crore of traded value, with effect from March 1, 2026</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>The exchange moved part of the charge out of the IPFT contribution; total outflow unchanged.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -659,6 +996,46 @@
           <t>NSE</t>
         </is>
       </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>futures</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2020-12-31</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0.000019</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>S25 existing Rs 1.90 each side per lakh (equity futures); S30 exchange txn charge 0.0019%</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Confirmed for 2018 to 2020 (Fyers calculator scripts, S31, S30) and for 2020-12-18 (NSE circular S25). The same rate is used back to 2010: earlier NSE rates and any ETF concessions were not researched.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -666,6 +1043,41 @@
           <t>NSE</t>
         </is>
       </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>futures</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2021-01-01</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2023-03-31</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0.00002</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>S25 revised Rs 2.00 each side per lakh, applicable with effect from January 01, 2021</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -673,6 +1085,41 @@
           <t>NSE</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>futures</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2023-04-01</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2024-03-31</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0.000019</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>S26 equity futures revised Rs 1.90 each side per lakh, applicable with effect from April 01, 2023</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -680,6 +1127,41 @@
           <t>NSE</t>
         </is>
       </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>futures</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2024-04-01</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2024-09-30</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0.0000188</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>S27 equity futures revised Rs 1.88 each side per lakh, applicable with effect from April 01, 2024</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -687,6 +1169,41 @@
           <t>NSE</t>
         </is>
       </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>futures</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2024-10-01</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0.0000173</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>S28 Equity Futures: Rs. 1.73 each side per lakh of traded value, with effect from October 1, 2024</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -699,8 +1216,10 @@
           <t>futures</t>
         </is>
       </c>
-      <c r="C13" s="2">
-        <v>46082</v>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -712,8 +1231,10 @@
           <t>S29 Equity futures transaction charges Rs. 182.99 each side per crore of traded value, with effect from March 1, 2026</t>
         </is>
       </c>
-      <c r="G13" s="2">
-        <v>46295</v>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -732,85 +1253,346 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>from</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>to</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>applies_to</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>verified_on</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
-        <v>40269</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2012-03-31</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>0.103</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>["brokerage", "exchange_txn", "clearing", "dp", "amc", "account_opening"]</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>S37 service tax 10.30% from 24 February 2009 to 31 March 2012</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Service tax, not GST. The rate is from S37; the taxed base (brokerage plus transaction charges) is assumed to match Fyers' GST-era base (S30), because no pre-2017 statement of the base was found.</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
-        <v>41000</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2012-04-01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2015-05-31</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>0.1236</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>["brokerage", "exchange_txn", "clearing", "dp", "amc", "account_opening"]</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>S37 service tax 12.36% from 1 April 2012 to 31 May 2015</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Service tax, not GST. The rate is from S37; the taxed base (brokerage plus transaction charges) is assumed to match Fyers' GST-era base (S30), because no pre-2017 statement of the base was found.</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2">
-        <v>42156</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2015-06-01</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2015-11-14</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>0.14</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>["brokerage", "exchange_txn", "clearing", "dp", "amc", "account_opening"]</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>S37 service tax 14% from 1 June 2015 to 14 November 2015</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Service tax, not GST. The rate is from S37; the taxed base (brokerage plus transaction charges) is assumed to match Fyers' GST-era base (S30), because no pre-2017 statement of the base was found.</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2">
-        <v>42323</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2015-11-15</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2016-05-31</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0.145</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>["brokerage", "exchange_txn", "clearing", "dp", "amc", "account_opening"]</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>S37 service tax 14.5% (14% + 0.5% Swachh Bharat Cess) from 15 November 2015 to 31 May 2016</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Service tax, not GST. The rate is from S37; the taxed base (brokerage plus transaction charges) is assumed to match Fyers' GST-era base (S30), because no pre-2017 statement of the base was found.</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2">
-        <v>42522</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2016-06-01</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2017-06-30</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>["brokerage", "exchange_txn", "clearing", "dp", "amc", "account_opening"]</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>S37 service tax 15% (14% + 0.5% + 0.5% Krishi Kalyan Cess) from 1 June 2016 to 30 June 2017</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Service tax, not GST. The rate is from S37; the taxed base (brokerage plus transaction charges) is assumed to match Fyers' GST-era base (S30), because no pre-2017 statement of the base was found.</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2">
-        <v>42917</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2017-07-01</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2023-06-04</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0.18</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>["brokerage", "exchange_txn", "clearing", "dp", "amc", "account_opening"]</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>S30 GST 18% on the value of brokerage and total transaction charges (exchange transaction and clearing member charges); S39 copy of 2022-01-24</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>GST from 1 July 2017.</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2">
-        <v>45082</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2023-06-05</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2025-03-16</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0.18</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>["brokerage", "exchange_txn", "clearing", "sebi", "dp", "amc", "account_opening"]</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>S39 GST 18% on (Brokerage + Exchange Transaction charges + Clearing charges + SEBI Turnover Fee), copy of 2023-06-05</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Date is the first archived copy showing the SEBI fee in the base; the copy of 2023-01-29 does not show it.</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2">
-        <v>45733</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2025-03-17</t>
+        </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -827,8 +1609,10 @@
           <t>S1 GST 18% on (Brokerage + Exchange Transaction charges + Clearing charges + SEBI Turnover Fee + NSE IPFT)</t>
         </is>
       </c>
-      <c r="F9" s="2">
-        <v>46295</v>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -852,47 +1636,47 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>exchange</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>segment</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>from</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>to</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>verified_on</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -904,6 +1688,46 @@
           <t>NSE</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>delivery</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2023-03-31</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0.000000001</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>S26 existing Rs.0.01 per crore of the traded value (as of 2023-03-24)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>The value is stated for March 2023 only; earlier values were not found. It is Rs 0.0001 per lakh, immaterial.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -911,6 +1735,46 @@
           <t>NSE</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>delivery</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2023-04-01</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.000001</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>S26 recalibrate the contribution to NSE IPFT from Rs.0.01 per crore to Rs.10 per crore of the traded value, from April 01, 2023; S29 confirms Rs. 10 each side</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Fyers' tables list it from March 2025 (S39).</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -918,6 +1782,36 @@
           <t>NSE</t>
         </is>
       </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>delivery</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.000000001</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>S29 contribution to NSE IPFT Rs. 0.01 each side per crore, with effect from March 1, 2026</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -925,6 +1819,46 @@
           <t>NSE</t>
         </is>
       </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>futures</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2023-03-31</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0.000000001</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>S26 existing Rs.0.01 per crore of the traded value (as of 2023-03-24)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>The value is stated for March 2023 only; earlier values were not found. It is Rs 0.0001 per lakh, immaterial.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -932,6 +1866,46 @@
           <t>NSE</t>
         </is>
       </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>futures</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2023-04-01</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.000001</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>S26 recalibrate the contribution to NSE IPFT from Rs.0.01 per crore to Rs.10 per crore of the traded value, from April 01, 2023; S29 confirms Rs. 10 each side</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Fyers' tables list it from March 2025 (S39).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -944,8 +1918,10 @@
           <t>futures</t>
         </is>
       </c>
-      <c r="C7" s="2">
-        <v>46082</v>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -957,8 +1933,10 @@
           <t>S29 contribution to NSE IPFT Rs. 0.01 each side per crore, with effect from March 1, 2026</t>
         </is>
       </c>
-      <c r="G7" s="2">
-        <v>46295</v>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -977,55 +1955,121 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>from</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>to</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>verified_on</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
-        <v>40269</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2017-03-31</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>0.000002</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>S34 broker turnover fee cut from Rs 20 to Rs 15 per crore in January 2017</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Rs 20 per crore before the cut; values for earlier years were not researched.</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
-        <v>42826</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2017-04-01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2019-03-31</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>0.0000015</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>S34 Rs 15 per crore after the January 2017 cut; S32 Board memorandum of March 2019: current fee Rs.15/- per crore; S31 0.00015% in 2018 and 2019</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Rs 15 per crore is confirmed for 2018 and 2019 (S31) and March 2019 (S32). The date of the January 2017 cut was not found, so 2017-04-01 is used.</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2">
-        <v>43556</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2019-04-01</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -1037,8 +2081,10 @@
           <t>S32 SEBI notification SEBI/LAD-NRO/GN/2019/03: 0.00010 per cent of turnover (Rs 10 per crore), in force from April 01, 2019</t>
         </is>
       </c>
-      <c r="E4" s="2">
-        <v>46295</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1062,47 +2108,47 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>segment</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>side</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>from</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>to</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>verified_on</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -1114,6 +2160,46 @@
           <t>delivery</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2020-06-30</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0.0001</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>S31 Maharashtra delivery stamp duty in Fyers' calculator</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>State-wise before 2020-07-01. Maharashtra is the default state: Fyers' calculator scripts of 2018 to 2020 (S31) list Maharashtra delivery 0.01% and futures 0.002%. Sellers also paid in some states; the engine charges the buy side only.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1121,6 +2207,41 @@
           <t>delivery</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2020-07-01</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.00015</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>S35 Transfer of security other than debenture on delivery basis 0.015% Buyer</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Uniform rate under the Indian Stamp Act amendments in force from 1 July 2020 (PIB, S35).</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1128,6 +2249,46 @@
           <t>delivery</t>
         </is>
       </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2020-06-30</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>S31 stamp duty on the buy side only in broker practice</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>State-wise before 2020-07-01. Maharashtra is the default state: Fyers' calculator scripts of 2018 to 2020 (S31) list Maharashtra delivery 0.01% and futures 0.002%. Sellers also paid in some states; the engine charges the buy side only.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1135,6 +2296,36 @@
           <t>delivery</t>
         </is>
       </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2020-07-01</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>S35 stamp duty is levied only on the buyer</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1142,6 +2333,46 @@
           <t>futures</t>
         </is>
       </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2020-06-30</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.00002</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>S31 Maharashtra futures stamp duty in Fyers' calculator</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>State-wise before 2020-07-01. Maharashtra is the default state: Fyers' calculator scripts of 2018 to 2020 (S31) list Maharashtra delivery 0.01% and futures 0.002%. Sellers also paid in some states; the engine charges the buy side only.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1149,6 +2380,41 @@
           <t>futures</t>
         </is>
       </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2020-07-01</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0.00002</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>S35 Derivatives - Equity Futures 0.002% Buyer</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Uniform rate under the Indian Stamp Act amendments in force from 1 July 2020 (PIB, S35).</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1156,6 +2422,46 @@
           <t>futures</t>
         </is>
       </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2020-06-30</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>S31 stamp duty on the buy side only in broker practice</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>State-wise before 2020-07-01. Maharashtra is the default state: Fyers' calculator scripts of 2018 to 2020 (S31) list Maharashtra delivery 0.01% and futures 0.002%. Sellers also paid in some states; the engine charges the buy side only.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1163,6 +2469,36 @@
           <t>futures</t>
         </is>
       </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2020-07-01</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>S35 stamp duty is levied only on the buyer</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1170,6 +2506,46 @@
           <t>mf</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2020-06-30</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>S36 stamp duty on mutual fund purchases starts with effect from 1 July 2020</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>None before that date.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1177,6 +2553,36 @@
           <t>mf</t>
         </is>
       </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2020-07-01</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0.00005</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>S36 0.005% of the net investment value on purchases (issue of units), with effect from July 1, 2020</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1184,6 +2590,41 @@
           <t>mf</t>
         </is>
       </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2020-06-30</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>S36 stamp duty applies to purchases, not redemptions</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1196,8 +2637,10 @@
           <t>sell</t>
         </is>
       </c>
-      <c r="C13" s="2">
-        <v>44013</v>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2020-07-01</t>
+        </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1209,8 +2652,10 @@
           <t>S36 stamp duty applies to purchases, not redemptions</t>
         </is>
       </c>
-      <c r="G13" s="2">
-        <v>46295</v>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1229,52 +2674,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>instrument_class</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>side</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>from</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>to</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>round_step</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>verified_on</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -1286,6 +2731,51 @@
           <t>etf_equity</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2012-06-30</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0.00125</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>S18 units of an equity oriented fund, delivery based: existing rate 0.125%; S71 and S80 memoranda propose no change to STT</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>The Finance Bill 2012 memorandum (S18) gives 0.125% as the existing rate in March 2012, and neither the Finance Bill 2010 (S71) nor the 2011 memorandum (S80) changes STT, so the rate stood at 0.125% from 2010-04-01 to 2012-06-30.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1293,6 +2783,46 @@
           <t>etf_equity</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2012-07-01</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2013-05-31</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>S18 proposed 0.1% from 1st July 2012; S19 existing 0.1% in Feb 2013</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1300,6 +2830,46 @@
           <t>etf_equity</t>
         </is>
       </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2013-06-01</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>S19 delivery based purchase of units of an equity oriented fund: Nil from 1st June 2013; S23 lists no purchase of such units</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>No STT on buying ETF units.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1307,6 +2877,51 @@
           <t>etf_equity</t>
         </is>
       </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2012-06-30</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0.00125</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>S18 units of an equity oriented fund, delivery based: existing rate 0.125%; S71 and S80 memoranda propose no change to STT</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>The Finance Bill 2012 memorandum (S18) gives 0.125% as the existing rate in March 2012, and neither the Finance Bill 2010 (S71) nor the 2011 memorandum (S80) changes STT, so the rate stood at 0.125% from 2010-04-01 to 2012-06-30.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1314,6 +2929,46 @@
           <t>etf_equity</t>
         </is>
       </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2012-07-01</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2013-05-31</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>S18 proposed 0.1% from 1st July 2012; S19 existing 0.1% in Feb 2013</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1321,6 +2976,46 @@
           <t>etf_equity</t>
         </is>
       </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2013-06-01</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0.00001</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>S19 delivery based sale of units of an equity oriented fund: 0.001% from 1st June 2013; S20 and S23 item 2A: 0.001% (No Change)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Unchanged through the Finance Acts of 2016, 2023, 2024 and 2026 (NSE circulars S20 to S23).</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1328,6 +3023,46 @@
           <t>mf_equity</t>
         </is>
       </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>S19 the taxable transactions listed are sales of units; subscription to a fund from the fund house is not one</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Buying units from the fund house carries no STT.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1335,6 +3070,51 @@
           <t>mf_equity</t>
         </is>
       </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2013-05-31</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0.0025</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>S19 sale of a unit of an equity oriented fund to the mutual fund: existing 0.25%</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Redemption.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1342,6 +3122,46 @@
           <t>mf_equity</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2013-06-01</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0.00001</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>S19 sale of a unit of an equity oriented fund to the mutual fund: 0.001% from 1st June 2013</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Redemption. No later change found (NSE circulars S20 to S23 cover exchange sales only).</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1349,6 +3169,46 @@
           <t>etf_gold</t>
         </is>
       </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>S23 the STT table lists equity shares, business trust units, equity oriented fund units and derivatives only</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Units that are not equity oriented (gold ETFs, debt and liquid funds) carry no STT.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1356,6 +3216,46 @@
           <t>etf_gold</t>
         </is>
       </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>S23 the STT table lists equity shares, business trust units, equity oriented fund units and derivatives only</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Units that are not equity oriented (gold ETFs, debt and liquid funds) carry no STT.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1363,6 +3263,46 @@
           <t>mf_debt</t>
         </is>
       </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>S23 the STT table lists equity shares, business trust units, equity oriented fund units and derivatives only</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Units that are not equity oriented (gold ETFs, debt and liquid funds) carry no STT.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1370,6 +3310,46 @@
           <t>mf_debt</t>
         </is>
       </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>S23 the STT table lists equity shares, business trust units, equity oriented fund units and derivatives only</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Units that are not equity oriented (gold ETFs, debt and liquid funds) carry no STT.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1377,6 +3357,41 @@
           <t>fut_index</t>
         </is>
       </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>S20 and S23: STT on a futures in securities is payable by the seller</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1384,6 +3399,46 @@
           <t>fut_index</t>
         </is>
       </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2013-05-31</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0.00017</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>S19 sale of a futures in securities: existing 0.017%</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1391,6 +3446,46 @@
           <t>fut_index</t>
         </is>
       </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2013-06-01</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2023-03-31</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>0.0001</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>S19 futures 0.01% from 1st June 2013; S20 futures 0.01 per cent (No Change) in 2016; S21 up to March 31, 2023: 0.01%</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1398,6 +3493,51 @@
           <t>fut_index</t>
         </is>
       </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2023-04-01</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2024-09-30</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>0.000125</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>S21 Sale of a futures in securities has been revised to 0.0125% (upto March 31, 2023 - 0.01%)</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Finance Act 2023.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1405,6 +3545,51 @@
           <t>fut_index</t>
         </is>
       </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2024-10-01</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>0.0002</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>S22 Sale of a futures in securities has been revised to 0.02% (upto September 30, 2024 - 0.0125%)</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Finance Act 2024.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1412,6 +3597,46 @@
           <t>fut_index</t>
         </is>
       </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>0.0005</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>S23 Sale of a futures in securities has been revised to 0.05% (upto March 31, 2026 - 0.02%)</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Finance Act 2026.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1419,6 +3644,51 @@
           <t>eq_share</t>
         </is>
       </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2012-06-30</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>0.00125</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>S18 delivery based purchase of an equity share: existing rate 0.125%, reduced to 0.1% from 1st July 2012</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Listed equity shares bought for delivery: STT on both sides, unlike ETF units.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1426,6 +3696,41 @@
           <t>eq_share</t>
         </is>
       </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2012-07-01</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>S18 0.1% from 1st July 2012; S23 delivery based purchase of an equity share: 0.1% (No Change)</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1433,6 +3738,46 @@
           <t>eq_share</t>
         </is>
       </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2010-04-01</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2012-06-30</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>0.00125</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>S18 delivery based sale of an equity share: existing rate 0.125%, reduced to 0.1% from 1st July 2012</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1445,8 +3790,10 @@
           <t>sell</t>
         </is>
       </c>
-      <c r="C24" s="2">
-        <v>41091</v>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2012-07-01</t>
+        </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1463,8 +3810,10 @@
           <t>S18 0.1% from 1st July 2012; S23 delivery based sale of an equity share: 0.1% (No Change)</t>
         </is>
       </c>
-      <c r="H24" s="2">
-        <v>46297</v>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>

</xml_diff>